<commit_message>
Update regression data compilation
</commit_message>
<xml_diff>
--- a/Data/distance_to_nodes.xlsx
+++ b/Data/distance_to_nodes.xlsx
@@ -7099,7 +7099,7 @@
         <v>841</v>
       </c>
       <c r="B843">
-        <v>21.42181156028578</v>
+        <v>19.65390851242243</v>
       </c>
     </row>
     <row r="844">
@@ -7107,7 +7107,7 @@
         <v>842</v>
       </c>
       <c r="B844">
-        <v>22.49522263623879</v>
+        <v>21.38233355225105</v>
       </c>
     </row>
     <row r="845">
@@ -7115,7 +7115,7 @@
         <v>843</v>
       </c>
       <c r="B845">
-        <v>16.19161085190039</v>
+        <v>13.8605616975647</v>
       </c>
     </row>
     <row r="846">
@@ -7123,7 +7123,7 @@
         <v>844</v>
       </c>
       <c r="B846">
-        <v>20.9797932727014</v>
+        <v>18.69497252898393</v>
       </c>
     </row>
     <row r="847">
@@ -7131,7 +7131,7 @@
         <v>845</v>
       </c>
       <c r="B847">
-        <v>16.72536110107141</v>
+        <v>14.80905044784205</v>
       </c>
     </row>
     <row r="848">
@@ -7139,7 +7139,7 @@
         <v>846</v>
       </c>
       <c r="B848">
-        <v>19.50172462641531</v>
+        <v>18.39870558878141</v>
       </c>
     </row>
     <row r="849">
@@ -7155,7 +7155,7 @@
         <v>848</v>
       </c>
       <c r="B850">
-        <v>24.16635132296783</v>
+        <v>21.9705101648932</v>
       </c>
     </row>
     <row r="851">
@@ -7163,7 +7163,7 @@
         <v>849</v>
       </c>
       <c r="B851">
-        <v>19.49520767934272</v>
+        <v>16.90481363442589</v>
       </c>
     </row>
     <row r="852">
@@ -7171,7 +7171,7 @@
         <v>850</v>
       </c>
       <c r="B852">
-        <v>23.65685581179383</v>
+        <v>21.68222116567546</v>
       </c>
     </row>
     <row r="853">
@@ -7187,7 +7187,7 @@
         <v>852</v>
       </c>
       <c r="B854">
-        <v>16.62252273937216</v>
+        <v>15.24053375330743</v>
       </c>
     </row>
     <row r="855">
@@ -7299,7 +7299,7 @@
         <v>866</v>
       </c>
       <c r="B868">
-        <v>6.801876198379063</v>
+        <v>6.306982972332919</v>
       </c>
     </row>
     <row r="869">
@@ -7307,7 +7307,7 @@
         <v>867</v>
       </c>
       <c r="B869">
-        <v>8.900894857005918</v>
+        <v>8.93959382185113</v>
       </c>
     </row>
     <row r="870">
@@ -7323,7 +7323,7 @@
         <v>869</v>
       </c>
       <c r="B871">
-        <v>11.96872854148653</v>
+        <v>10.91660469586549</v>
       </c>
     </row>
     <row r="872">
@@ -7347,7 +7347,7 @@
         <v>872</v>
       </c>
       <c r="B874">
-        <v>18.27377477470923</v>
+        <v>18.6967397880025</v>
       </c>
     </row>
     <row r="875">
@@ -7363,7 +7363,7 @@
         <v>874</v>
       </c>
       <c r="B876">
-        <v>17.87428310803395</v>
+        <v>17.3803224755321</v>
       </c>
     </row>
     <row r="877">
@@ -7371,7 +7371,7 @@
         <v>875</v>
       </c>
       <c r="B877">
-        <v>14.70861967983075</v>
+        <v>14.11035630506033</v>
       </c>
     </row>
     <row r="878">
@@ -7379,7 +7379,7 @@
         <v>876</v>
       </c>
       <c r="B878">
-        <v>14.56119732156985</v>
+        <v>14.55254208396978</v>
       </c>
     </row>
     <row r="879">
@@ -7403,7 +7403,7 @@
         <v>879</v>
       </c>
       <c r="B881">
-        <v>11.0455365572774</v>
+        <v>10.78900252384516</v>
       </c>
     </row>
     <row r="882">
@@ -7827,7 +7827,7 @@
         <v>932</v>
       </c>
       <c r="B934">
-        <v>14.80921083333351</v>
+        <v>15.49414830618528</v>
       </c>
     </row>
     <row r="935">
@@ -7851,7 +7851,7 @@
         <v>935</v>
       </c>
       <c r="B937">
-        <v>13.41104083002249</v>
+        <v>14.1694078138738</v>
       </c>
     </row>
     <row r="938">
@@ -7867,7 +7867,7 @@
         <v>937</v>
       </c>
       <c r="B939">
-        <v>6.479186244217921</v>
+        <v>7.593248007981491</v>
       </c>
     </row>
     <row r="940">
@@ -7907,7 +7907,7 @@
         <v>942</v>
       </c>
       <c r="B944">
-        <v>9.316722992772174</v>
+        <v>11.03624346950976</v>
       </c>
     </row>
     <row r="945">
@@ -7915,7 +7915,7 @@
         <v>943</v>
       </c>
       <c r="B945">
-        <v>12.42437791206936</v>
+        <v>13.20512845698603</v>
       </c>
     </row>
     <row r="946">
@@ -8099,7 +8099,7 @@
         <v>966</v>
       </c>
       <c r="B968">
-        <v>11.85630293528173</v>
+        <v>8.920214792607071</v>
       </c>
     </row>
     <row r="969">
@@ -8107,7 +8107,7 @@
         <v>967</v>
       </c>
       <c r="B969">
-        <v>14.72806652491029</v>
+        <v>11.82964498135253</v>
       </c>
     </row>
     <row r="970">
@@ -8115,7 +8115,7 @@
         <v>968</v>
       </c>
       <c r="B970">
-        <v>16.65318338247413</v>
+        <v>14.12211206864431</v>
       </c>
     </row>
     <row r="971">
@@ -8123,7 +8123,7 @@
         <v>969</v>
       </c>
       <c r="B971">
-        <v>4.329742754778716</v>
+        <v>1.714410359024305</v>
       </c>
     </row>
     <row r="972">
@@ -8131,7 +8131,7 @@
         <v>970</v>
       </c>
       <c r="B972">
-        <v>12.06107822984307</v>
+        <v>9.985674461536117</v>
       </c>
     </row>
     <row r="973">
@@ -8139,7 +8139,7 @@
         <v>971</v>
       </c>
       <c r="B973">
-        <v>12.17875737154927</v>
+        <v>9.511204507116107</v>
       </c>
     </row>
     <row r="974">
@@ -8147,7 +8147,7 @@
         <v>972</v>
       </c>
       <c r="B974">
-        <v>12.53525088308245</v>
+        <v>9.812459017599531</v>
       </c>
     </row>
     <row r="975">
@@ -8155,7 +8155,7 @@
         <v>973</v>
       </c>
       <c r="B975">
-        <v>9.936982722872296</v>
+        <v>7.16712873994878</v>
       </c>
     </row>
     <row r="976">
@@ -8163,7 +8163,7 @@
         <v>974</v>
       </c>
       <c r="B976">
-        <v>13.10914744244024</v>
+        <v>10.8776215075781</v>
       </c>
     </row>
     <row r="977">
@@ -8171,7 +8171,7 @@
         <v>975</v>
       </c>
       <c r="B977">
-        <v>6.57723881833802</v>
+        <v>4.232436656350789</v>
       </c>
     </row>
     <row r="978">
@@ -8179,7 +8179,7 @@
         <v>976</v>
       </c>
       <c r="B978">
-        <v>17.35910146690644</v>
+        <v>14.51391367471693</v>
       </c>
     </row>
     <row r="979">
@@ -8187,7 +8187,7 @@
         <v>977</v>
       </c>
       <c r="B979">
-        <v>8.176936501283164</v>
+        <v>5.509956006905899</v>
       </c>
     </row>
     <row r="980">
@@ -8195,7 +8195,7 @@
         <v>978</v>
       </c>
       <c r="B980">
-        <v>8.420116806889435</v>
+        <v>6.602531664937675</v>
       </c>
     </row>
     <row r="981">
@@ -8203,7 +8203,7 @@
         <v>979</v>
       </c>
       <c r="B981">
-        <v>23.19789886850822</v>
+        <v>25.52254620683486</v>
       </c>
     </row>
     <row r="982">
@@ -8211,7 +8211,7 @@
         <v>980</v>
       </c>
       <c r="B982">
-        <v>19.56498261687737</v>
+        <v>22.09045143432118</v>
       </c>
     </row>
     <row r="983">
@@ -8219,7 +8219,7 @@
         <v>981</v>
       </c>
       <c r="B983">
-        <v>18.05641778626574</v>
+        <v>20.0478210117097</v>
       </c>
     </row>
     <row r="984">
@@ -8227,7 +8227,7 @@
         <v>982</v>
       </c>
       <c r="B984">
-        <v>15.44800993660738</v>
+        <v>18.12300782455958</v>
       </c>
     </row>
     <row r="985">
@@ -8235,7 +8235,7 @@
         <v>983</v>
       </c>
       <c r="B985">
-        <v>21.87330052677519</v>
+        <v>22.58286726743913</v>
       </c>
     </row>
     <row r="986">
@@ -8243,7 +8243,7 @@
         <v>984</v>
       </c>
       <c r="B986">
-        <v>15.33930621141995</v>
+        <v>17.50685840717249</v>
       </c>
     </row>
     <row r="987">
@@ -8251,7 +8251,7 @@
         <v>985</v>
       </c>
       <c r="B987">
-        <v>21.39926964535066</v>
+        <v>23.57932037443232</v>
       </c>
     </row>
     <row r="988">
@@ -8259,7 +8259,7 @@
         <v>986</v>
       </c>
       <c r="B988">
-        <v>26.62559967475715</v>
+        <v>28.66150841427597</v>
       </c>
     </row>
     <row r="989">
@@ -8347,7 +8347,7 @@
         <v>997</v>
       </c>
       <c r="B999">
-        <v>12.10556502925399</v>
+        <v>12.57761939936718</v>
       </c>
     </row>
     <row r="1000">
@@ -8363,7 +8363,7 @@
         <v>999</v>
       </c>
       <c r="B1001">
-        <v>12.82521446296451</v>
+        <v>14.59799581025459</v>
       </c>
     </row>
     <row r="1002">
@@ -8379,7 +8379,7 @@
         <v>1001</v>
       </c>
       <c r="B1003">
-        <v>11.92766163079851</v>
+        <v>14.60382992552079</v>
       </c>
     </row>
     <row r="1004">
@@ -8387,7 +8387,7 @@
         <v>1002</v>
       </c>
       <c r="B1004">
-        <v>10.5246677954652</v>
+        <v>12.83429868554952</v>
       </c>
     </row>
     <row r="1005">
@@ -8395,7 +8395,7 @@
         <v>1003</v>
       </c>
       <c r="B1005">
-        <v>8.823289604887609</v>
+        <v>11.30404102117589</v>
       </c>
     </row>
     <row r="1006">
@@ -8403,7 +8403,7 @@
         <v>1004</v>
       </c>
       <c r="B1006">
-        <v>8.845700007249018</v>
+        <v>11.7685686957084</v>
       </c>
     </row>
     <row r="1007">
@@ -8507,7 +8507,7 @@
         <v>1017</v>
       </c>
       <c r="B1019">
-        <v>21.77838752035956</v>
+        <v>22.8850024213061</v>
       </c>
     </row>
     <row r="1020">
@@ -8515,7 +8515,7 @@
         <v>1018</v>
       </c>
       <c r="B1020">
-        <v>18.87627066174108</v>
+        <v>20.3678326598375</v>
       </c>
     </row>
     <row r="1021">
@@ -8523,7 +8523,7 @@
         <v>1019</v>
       </c>
       <c r="B1021">
-        <v>21.86754100069239</v>
+        <v>23.56948507444276</v>
       </c>
     </row>
     <row r="1022">
@@ -8531,7 +8531,7 @@
         <v>1020</v>
       </c>
       <c r="B1022">
-        <v>5.895271467174473</v>
+        <v>8.727620073462889</v>
       </c>
     </row>
     <row r="1023">
@@ -8539,7 +8539,7 @@
         <v>1021</v>
       </c>
       <c r="B1023">
-        <v>4.926288307002339</v>
+        <v>6.7385465457903</v>
       </c>
     </row>
     <row r="1024">
@@ -8547,7 +8547,7 @@
         <v>1022</v>
       </c>
       <c r="B1024">
-        <v>8.315523484891372</v>
+        <v>10.43366744837717</v>
       </c>
     </row>
     <row r="1025">
@@ -8555,7 +8555,7 @@
         <v>1023</v>
       </c>
       <c r="B1025">
-        <v>5.349276700650416</v>
+        <v>8.118944230188216</v>
       </c>
     </row>
     <row r="1026">
@@ -8563,7 +8563,7 @@
         <v>1024</v>
       </c>
       <c r="B1026">
-        <v>7.111332213750659</v>
+        <v>9.508648129013466</v>
       </c>
     </row>
     <row r="1027">
@@ -8571,7 +8571,7 @@
         <v>1025</v>
       </c>
       <c r="B1027">
-        <v>22.22504355744513</v>
+        <v>21.64950372652624</v>
       </c>
     </row>
     <row r="1028">
@@ -8579,7 +8579,7 @@
         <v>1026</v>
       </c>
       <c r="B1028">
-        <v>7.624815221760368</v>
+        <v>7.100262537981658</v>
       </c>
     </row>
     <row r="1029">
@@ -8595,7 +8595,7 @@
         <v>1028</v>
       </c>
       <c r="B1030">
-        <v>22.66979779760182</v>
+        <v>21.19002101561528</v>
       </c>
     </row>
     <row r="1031">
@@ -8603,7 +8603,7 @@
         <v>1029</v>
       </c>
       <c r="B1031">
-        <v>12.14410868371082</v>
+        <v>10.89683881179044</v>
       </c>
     </row>
     <row r="1032">
@@ -8611,7 +8611,7 @@
         <v>1030</v>
       </c>
       <c r="B1032">
-        <v>3.829650916653252</v>
+        <v>2.699337278754647</v>
       </c>
     </row>
     <row r="1033">
@@ -8619,7 +8619,7 @@
         <v>1031</v>
       </c>
       <c r="B1033">
-        <v>19.69633273063405</v>
+        <v>17.74704956858763</v>
       </c>
     </row>
     <row r="1034">
@@ -8627,7 +8627,7 @@
         <v>1032</v>
       </c>
       <c r="B1034">
-        <v>17.98165975846372</v>
+        <v>16.55203774469037</v>
       </c>
     </row>
     <row r="1035">
@@ -8643,7 +8643,7 @@
         <v>1034</v>
       </c>
       <c r="B1036">
-        <v>13.81844086345078</v>
+        <v>12.10016086527797</v>
       </c>
     </row>
     <row r="1037">
@@ -8659,7 +8659,7 @@
         <v>1036</v>
       </c>
       <c r="B1038">
-        <v>16.72578789112604</v>
+        <v>14.41183207715983</v>
       </c>
     </row>
     <row r="1039">
@@ -8667,7 +8667,7 @@
         <v>1037</v>
       </c>
       <c r="B1039">
-        <v>18.22407726798037</v>
+        <v>16.52803447182866</v>
       </c>
     </row>
     <row r="1040">
@@ -8675,7 +8675,7 @@
         <v>1038</v>
       </c>
       <c r="B1040">
-        <v>18.83164021078667</v>
+        <v>16.60646821359574</v>
       </c>
     </row>
     <row r="1041">
@@ -8683,7 +8683,7 @@
         <v>1039</v>
       </c>
       <c r="B1041">
-        <v>20.15032488589116</v>
+        <v>20.16734568436619</v>
       </c>
     </row>
     <row r="1042">
@@ -8691,7 +8691,7 @@
         <v>1040</v>
       </c>
       <c r="B1042">
-        <v>16.95529327165244</v>
+        <v>15.77590722418053</v>
       </c>
     </row>
     <row r="1043">
@@ -8699,7 +8699,7 @@
         <v>1041</v>
       </c>
       <c r="B1043">
-        <v>25.76042506694605</v>
+        <v>26.00889933028632</v>
       </c>
     </row>
     <row r="1044">
@@ -8707,7 +8707,7 @@
         <v>1042</v>
       </c>
       <c r="B1044">
-        <v>19.89665323387234</v>
+        <v>18.88729517883474</v>
       </c>
     </row>
     <row r="1045">
@@ -8715,7 +8715,7 @@
         <v>1043</v>
       </c>
       <c r="B1045">
-        <v>9.014944674336999</v>
+        <v>7.091951068546098</v>
       </c>
     </row>
     <row r="1046">
@@ -8755,7 +8755,7 @@
         <v>1048</v>
       </c>
       <c r="B1050">
-        <v>17.8817238953763</v>
+        <v>17.34808611312392</v>
       </c>
     </row>
     <row r="1051">
@@ -9147,7 +9147,7 @@
         <v>1097</v>
       </c>
       <c r="B1099">
-        <v>16.22498622328425</v>
+        <v>13.30534833739332</v>
       </c>
     </row>
     <row r="1100">
@@ -9155,7 +9155,7 @@
         <v>1098</v>
       </c>
       <c r="B1100">
-        <v>18.16659459177931</v>
+        <v>16.59293432232049</v>
       </c>
     </row>
     <row r="1101">
@@ -9171,7 +9171,7 @@
         <v>1100</v>
       </c>
       <c r="B1102">
-        <v>15.65848541488306</v>
+        <v>12.91066863426261</v>
       </c>
     </row>
     <row r="1103">
@@ -9187,7 +9187,7 @@
         <v>1102</v>
       </c>
       <c r="B1104">
-        <v>19.16414331284514</v>
+        <v>16.33895280646302</v>
       </c>
     </row>
     <row r="1105">
@@ -9283,7 +9283,7 @@
         <v>1114</v>
       </c>
       <c r="B1116">
-        <v>23.250410214744</v>
+        <v>21.58432581591429</v>
       </c>
     </row>
     <row r="1117">
@@ -9315,7 +9315,7 @@
         <v>1118</v>
       </c>
       <c r="B1120">
-        <v>26.29896998594824</v>
+        <v>24.45335495349909</v>
       </c>
     </row>
     <row r="1121">
@@ -9331,7 +9331,7 @@
         <v>1120</v>
       </c>
       <c r="B1122">
-        <v>25.26335813791615</v>
+        <v>25.10865721582872</v>
       </c>
     </row>
     <row r="1123">
@@ -12955,7 +12955,7 @@
         <v>1573</v>
       </c>
       <c r="B1575">
-        <v>3.754579480593483</v>
+        <v>5.171387257630506</v>
       </c>
     </row>
     <row r="1576">
@@ -13507,7 +13507,7 @@
         <v>1642</v>
       </c>
       <c r="B1644">
-        <v>2.028806557049571</v>
+        <v>4.963108320108936</v>
       </c>
     </row>
     <row r="1645">
@@ -13515,7 +13515,7 @@
         <v>1643</v>
       </c>
       <c r="B1645">
-        <v>0.833576887307609</v>
+        <v>2.594152426327075</v>
       </c>
     </row>
     <row r="1646">
@@ -13579,7 +13579,7 @@
         <v>1651</v>
       </c>
       <c r="B1653">
-        <v>26.43306470539659</v>
+        <v>28.45283509252831</v>
       </c>
     </row>
     <row r="1654">
@@ -13859,7 +13859,7 @@
         <v>1686</v>
       </c>
       <c r="B1688">
-        <v>16.98545211061418</v>
+        <v>19.21885102017499</v>
       </c>
     </row>
     <row r="1689">
@@ -13867,7 +13867,7 @@
         <v>1687</v>
       </c>
       <c r="B1689">
-        <v>15.62023236319789</v>
+        <v>16.82963245067203</v>
       </c>
     </row>
     <row r="1690">
@@ -13875,7 +13875,7 @@
         <v>1688</v>
       </c>
       <c r="B1690">
-        <v>8.213200592680051</v>
+        <v>9.188856624135081</v>
       </c>
     </row>
     <row r="1691">
@@ -13883,7 +13883,7 @@
         <v>1689</v>
       </c>
       <c r="B1691">
-        <v>12.38057977901964</v>
+        <v>14.02844543013261</v>
       </c>
     </row>
     <row r="1692">
@@ -13891,7 +13891,7 @@
         <v>1690</v>
       </c>
       <c r="B1692">
-        <v>17.2757676515808</v>
+        <v>16.82875973704438</v>
       </c>
     </row>
     <row r="1693">
@@ -13899,7 +13899,7 @@
         <v>1691</v>
       </c>
       <c r="B1693">
-        <v>13.32526951047298</v>
+        <v>15.40550577448183</v>
       </c>
     </row>
     <row r="1694">
@@ -13907,7 +13907,7 @@
         <v>1692</v>
       </c>
       <c r="B1694">
-        <v>18.65574960613958</v>
+        <v>19.28709925683625</v>
       </c>
     </row>
     <row r="1695">
@@ -13915,7 +13915,7 @@
         <v>1693</v>
       </c>
       <c r="B1695">
-        <v>10.51959486270761</v>
+        <v>12.02524259887938</v>
       </c>
     </row>
     <row r="1696">
@@ -13923,7 +13923,7 @@
         <v>1694</v>
       </c>
       <c r="B1696">
-        <v>12.01440772142921</v>
+        <v>11.75283238724364</v>
       </c>
     </row>
     <row r="1697">

</xml_diff>